<commit_message>
page-tags: other spellings move from Tags to Search aliases (Laozi, Zhuangzi, Mencius), so they never show as 'Also about'; backup of the sheet before the change
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/page-tags.xlsx
+++ b/content/page-tags.xlsx
@@ -1779,12 +1779,12 @@
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>Lao Tzŭ, Laotse, Tao Te Ching</t>
+          <t>Tao Te Ching</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>Lao Tzu</t>
+          <t>Lao Tzu, Lao Tzŭ, Laotse</t>
         </is>
       </c>
     </row>
@@ -1907,7 +1907,7 @@
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>Mengzi, human nature</t>
+          <t>human nature</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
@@ -2327,12 +2327,12 @@
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>great knowledge, the useless tree, Chuang Tzŭ</t>
+          <t>great knowledge, the useless tree</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>Chuang Tzu</t>
+          <t>Chuang Tzu, Chuang Tzŭ</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Library: Related for all 56 paths, eras, and topics; keywords reordered
page-related.xlsx: up to 6 related pages per path, era, and topic (paths
start with their best-known thinker; eras don't repeat their own thinkers).
page-tags.xlsx: most telling keywords first on every page (works first for
thinkers, places and events for eras, no title words for topics); the four
concept pages' doc tags reordered to match; "Enlightenment" removed from the
Enlightenment Ethics search aliases so the era is no longer linked to the path.
Checked with build_pages.py on a copy: every Related name resolves.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XtUBtsHEVvdoDDiuP88LhW
</commit_message>
<xml_diff>
--- a/content/page-tags.xlsx
+++ b/content/page-tags.xlsx
@@ -511,7 +511,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>America, United States, Transcendentalism, abolition</t>
+          <t>United States, Transcendentalism, slavery, abolition, Civil War, Seneca Falls</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr"/>
@@ -529,7 +529,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Athens, ancient Greece, Greeks, classical antiquity</t>
+          <t>Athens, city-states, classical antiquity, Hellenistic, Greeks</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr"/>
@@ -547,7 +547,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>ancient India, Vedas, Buddha, shramanas</t>
+          <t>Vedas, Buddha, shramanas, caste, Indo-Greeks</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr"/>
@@ -565,7 +565,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>colonialism, British India, Meiji Japan, East and West</t>
+          <t>colonialism, British India, Meiji Japan, East and West, Parliament of Religions</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr"/>
@@ -583,7 +583,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>ancient China, Warring States, Zhou, Hundred Schools</t>
+          <t>Warring States, Zhou dynasty, Qin, Hundred Schools, Mandate of Heaven, ancient China</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr"/>
@@ -601,7 +601,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>19th century, Industrial Revolution, Russia, Victorian</t>
+          <t>Industrial Revolution, 1848, serfdom, Victorian, Darwin</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr"/>
@@ -619,7 +619,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>17th century, Thirty Years' War, Scientific Revolution, wars of religion</t>
+          <t>Thirty Years' War, Scientific Revolution, wars of religion, English Civil War, Galileo</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
@@ -637,7 +637,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>world wars, 20th century, First World War, Second World War, Holocaust</t>
+          <t>First World War, Second World War, Holocaust, 20th century, world wars</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
@@ -655,7 +655,7 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Heian, Kamakura, samurai, medieval Japan</t>
+          <t>Heian, Kamakura, samurai, court women, mappō, medieval Japan</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
@@ -673,7 +673,7 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Renaissance, humanism, Reformation, Black Death</t>
+          <t>humanism, Black Death, printing, Reformation, Florence, wars of religion</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
@@ -691,7 +691,7 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Rome, Roman Empire, Romans, antiquity</t>
+          <t>Roman Empire, Augustus, Pax Romana, slavery, Christianity, Romans</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
@@ -709,7 +709,7 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Enlightenment, Age of Reason, 18th century, philosophes</t>
+          <t>Age of Reason, 18th century, philosophes, salons, Encyclopédie, slave trade</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr"/>
@@ -727,7 +727,7 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Islamic world, Persia, Baghdad, Islamic Golden Age, Mongols</t>
+          <t>Baghdad, Persia, Seljuks, Mongols, Islamic Golden Age, Sufis</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr"/>
@@ -745,7 +745,7 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>history, context, history of mentalities</t>
+          <t>history of mentalities, history, context</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr"/>
@@ -763,7 +763,7 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Buddhism, Buddha, nirvana, mindfulness</t>
+          <t>Buddha, nirvana, not-self, mindfulness, Dhamma, impermanence</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -785,7 +785,7 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>ancient Greek philosophy, Socrates, virtue, eudaimonia</t>
+          <t>Socrates, eudaimonia, virtue, the soul, Athens</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -807,7 +807,7 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>ritual, filial piety, junzi, the Way</t>
+          <t>junzi, ren, ritual, filial piety, Analects, the mean</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -829,12 +829,12 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Enlightenment, reason, rights, utilitarianism</t>
+          <t>Enlightenment, reason, rights, utilitarianism, categorical imperative, social contract</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Enlightenment, Utilitarianism, utilitarian</t>
+          <t>Utilitarianism, utilitarian</t>
         </is>
       </c>
     </row>
@@ -851,7 +851,7 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>pleasure, ataraxia, friendship, atoms</t>
+          <t>ataraxia, pleasure, the Garden, atoms, friendship</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -873,7 +873,7 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>existentialism, meaning, anxiety, the absurd</t>
+          <t>existentialism, meaning, anxiety, the absurd, God is dead</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -895,7 +895,7 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>humanism, essays, Renaissance, moralists</t>
+          <t>humanism, essays, moralists, maxims, Renaissance, Transcendentalism</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -917,7 +917,7 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Hinduism, Vedanta, Upanishads, yoga</t>
+          <t>Vedanta, Atman, Brahman, karma, dharma, yoga, Hinduism</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -939,7 +939,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>emptiness, imperfection, seasons, wabi-sabi, mono no aware, tea ceremony, Zen</t>
+          <t>wabi-sabi, mono no aware, tea ceremony, Zen, imperfection, emptiness, seasons</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr"/>
@@ -957,7 +957,7 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>heart, divine love, halting-station, wine, Sufism, mysticism, ghazal</t>
+          <t>Sufism, divine love, ghazal, mysticism, nafs, wine, heart, halting-station</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -979,7 +979,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>tranquillity, Stoics, virtue, what is in our control, resilience</t>
+          <t>what is in our control, virtue, tranquillity, resilience, memento mori, Stoics</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -1001,7 +1001,7 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>softness, water, Tao, the Way, wu wei</t>
+          <t>Tao, wu wei, the Way, water, softness, emptiness</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -1023,7 +1023,7 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>non-attachment</t>
+          <t>Krishna, Arjuna, non-attachment, karma yoga, svadharma</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -1045,7 +1045,7 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>the wise</t>
+          <t>the Buddha, the wise, Dhamma</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -1067,7 +1067,7 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Nagasena</t>
+          <t>Nagasena, Menander, the chariot</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -1089,7 +1089,7 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Katha Upanishad, Isha Upanishad, Brihadaranyaka Upanishad, Mundaka Upanishad</t>
+          <t>Atman, Brahman, Katha Upanishad, Isha Upanishad, Brihadaranyaka Upanishad, Mundaka Upanishad</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -1111,7 +1111,7 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>sympathy, The Theory of Moral Sentiments</t>
+          <t>The Theory of Moral Sentiments, The Wealth of Nations, sympathy</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr"/>
@@ -1169,7 +1169,7 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>boredom, Parerga and Paralipomena</t>
+          <t>Parerga and Paralipomena, boredom, pessimism, the will</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -1213,7 +1213,7 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>diversion, the heart's reasons, Pensées</t>
+          <t>Pensées, the heart's reasons, diversion</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -1253,7 +1253,7 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>mean man, superior man, reciprocity, the mean, Analects</t>
+          <t>Analects, superior man, reciprocity, the mean, ren, mean man</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>custom, A Treatise of Human Nature, An Enquiry Concerning Human Understanding</t>
+          <t>A Treatise of Human Nature, An Enquiry Concerning Human Understanding, custom, bundle of perceptions</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -1297,7 +1297,7 @@
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Diderot effect, Philosophical Thoughts, Regrets on My Old Dressing Gown</t>
+          <t>Encyclopédie, Philosophical Thoughts, Regrets on My Old Dressing Gown, Diderot effect</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
@@ -1319,7 +1319,7 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Discourse on Happiness</t>
+          <t>Discourse on Happiness, Newton's Principia, physics</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
@@ -1363,7 +1363,7 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Discourses, Enchiridion</t>
+          <t>Enchiridion, Discourses, what is in our power</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr"/>
@@ -1381,7 +1381,7 @@
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>The Garden, Principal Doctrines, Letter to Menoeceus, Vatican Sayings</t>
+          <t>Letter to Menoeceus, Principal Doctrines, The Garden, Vatican Sayings, ataraxia, pleasure</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr"/>
@@ -1439,7 +1439,7 @@
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>become who you are, Thus Spake Zarathustra, Beyond Good and Evil, The Joyful Wisdom, Human, All Too Human</t>
+          <t>Thus Spake Zarathustra, Beyond Good and Evil, become who you are, God is dead, The Joyful Wisdom, Human, All Too Human</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
@@ -1461,7 +1461,7 @@
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>active love, self-deception, The Brothers Karamazov, Notes from Underground</t>
+          <t>The Brothers Karamazov, Notes from Underground, Crime and Punishment, active love, self-deception</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
@@ -1545,7 +1545,7 @@
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>daimon</t>
+          <t>fragments, everything flows, daimon, Logos</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr"/>
@@ -1585,7 +1585,7 @@
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>moral law, good will, respect, Groundwork, Critique of Practical Reason</t>
+          <t>Groundwork, Critique of Practical Reason, categorical imperative, moral law, good will, respect</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
@@ -1673,7 +1673,7 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>Mill's Autobiography, On Liberty</t>
+          <t>On Liberty, Utilitarianism, The Subjection of Women, Mill's Autobiography, harm principle</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
@@ -1757,7 +1757,7 @@
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>maxim</t>
+          <t>Maxims, self-love, moralists, maxim</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
@@ -1779,7 +1779,7 @@
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>Tao Te Ching</t>
+          <t>Tao Te Ching, wu wei, the Way</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
@@ -1907,7 +1907,7 @@
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>human nature</t>
+          <t>human nature, righteousness, the people first</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
@@ -2039,7 +2039,7 @@
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>Laws, Apology, Socratic wisdom, Socrates, Crito, Phaedo, Republic, Symposium, Phaedrus, Gorgias, Theaetetus, Meno</t>
+          <t>Republic, Apology, Symposium, Phaedo, Socrates, Socratic wisdom, Laws, Crito, Phaedrus, Gorgias, Theaetetus, Meno</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr"/>
@@ -2079,7 +2079,7 @@
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>self-reliance, Self-Reliance, Nature</t>
+          <t>Self-Reliance, Nature, Transcendentalism</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
@@ -2207,7 +2207,7 @@
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>attention</t>
+          <t>The Need for Roots, attention, Gravity and Grace, factory work</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
@@ -2251,7 +2251,7 @@
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>commonwealth, Leviathan</t>
+          <t>Leviathan, commonwealth, social contract, state of nature</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
@@ -2291,7 +2291,7 @@
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>citizen of the world, Candide, Zadig, Philosophical Dictionary</t>
+          <t>Candide, Philosophical Dictionary, Zadig, citizen of the world, tolerance</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr"/>
@@ -2327,7 +2327,7 @@
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>great knowledge, the useless tree</t>
+          <t>the useless tree, great knowledge, butterfly dream</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
@@ -2349,7 +2349,7 @@
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>beauty, art, aesthetics, taste</t>
+          <t>aesthetics, taste, wabi-sabi, imperfection, the beautiful</t>
         </is>
       </c>
       <c r="D91" s="2" t="inlineStr"/>
@@ -2367,7 +2367,7 @@
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>change, impermanence, transience, flux</t>
+          <t>transience, flux, mono no aware, everything passes</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr"/>
@@ -2385,7 +2385,7 @@
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>character, virtue, integrity, junzi, gentleman</t>
+          <t>integrity, junzi, superior man, moral character, honesty</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr"/>
@@ -2403,7 +2403,7 @@
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>death, mortality, dying, grief, memento mori</t>
+          <t>dying, grief, memento mori, afterlife, fear of death</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr"/>
@@ -2421,7 +2421,7 @@
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>democracy, voting, citizens, government</t>
+          <t>voting, the people, citizens, majority rule, self-government</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr"/>
@@ -2439,7 +2439,7 @@
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>craving, desire, simplicity, wanting less, possessions, contentment</t>
+          <t>craving, wanting less, contentment, non-attachment, possessions, frugality</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr"/>
@@ -2455,11 +2455,7 @@
           <t>Duty</t>
         </is>
       </c>
-      <c r="C97" s="2" t="inlineStr">
-        <is>
-          <t>duty</t>
-        </is>
-      </c>
+      <c r="C97" s="2" t="n"/>
       <c r="D97" s="2" t="inlineStr"/>
     </row>
     <row r="98">
@@ -2475,7 +2471,7 @@
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>ego, pride, humility, vanity, self-love</t>
+          <t>vanity, self-love, arrogance, modesty, self-conceit</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr"/>
@@ -2493,7 +2489,7 @@
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>equality, inequality, fairness, women's rights</t>
+          <t>inequality, fairness, women's rights, natural rights, class</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr"/>
@@ -2509,11 +2505,7 @@
           <t>Fortune</t>
         </is>
       </c>
-      <c r="C100" s="2" t="inlineStr">
-        <is>
-          <t>fortune, what is in our power</t>
-        </is>
-      </c>
+      <c r="C100" s="2" t="n"/>
       <c r="D100" s="2" t="inlineStr"/>
     </row>
     <row r="101">
@@ -2529,7 +2521,7 @@
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>liberty, individuality, freedom, free will, choice, autonomy</t>
+          <t>liberty, free will, individuality, choice, autonomy, inner freedom</t>
         </is>
       </c>
       <c r="D101" s="2" t="inlineStr"/>
@@ -2547,7 +2539,7 @@
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>friendship, friends, kindness, compassion</t>
+          <t>friends, compassion, generosity, benevolence, ren</t>
         </is>
       </c>
       <c r="D102" s="2" t="inlineStr"/>
@@ -2565,7 +2557,7 @@
       </c>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>habit, practice, discipline, routine</t>
+          <t>discipline, routine, training, repetition, self-discipline</t>
         </is>
       </c>
       <c r="D103" s="2" t="inlineStr"/>
@@ -2583,7 +2575,7 @@
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>pleasure, happiness, the good life, eudaimonia, flourishing, wellbeing</t>
+          <t>pleasure, eudaimonia, flourishing, contentment, wellbeing, joy</t>
         </is>
       </c>
       <c r="D104" s="2" t="inlineStr"/>
@@ -2601,7 +2593,7 @@
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>social contract, justice, injustice, power, leadership</t>
+          <t>power, leadership, injustice, social contract, rulers, fairness</t>
         </is>
       </c>
       <c r="D105" s="2" t="inlineStr"/>
@@ -2617,7 +2609,7 @@
           <t>Karma and dharma</t>
         </is>
       </c>
-      <c r="C106" s="2" t="inlineStr"/>
+      <c r="C106" s="2" t="n"/>
       <c r="D106" s="2" t="inlineStr"/>
     </row>
     <row r="107">
@@ -2633,7 +2625,7 @@
       </c>
       <c r="C107" s="2" t="inlineStr">
         <is>
-          <t>law, rights, human rights, authority</t>
+          <t>human rights, natural rights, authority, rule of law, social contract</t>
         </is>
       </c>
       <c r="D107" s="2" t="inlineStr"/>
@@ -2651,7 +2643,7 @@
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>learning, knowledge, education, wisdom, truth</t>
+          <t>education, wisdom, truth, ignorance, study, curiosity</t>
         </is>
       </c>
       <c r="D108" s="2" t="inlineStr"/>
@@ -2669,7 +2661,7 @@
       </c>
       <c r="C109" s="2" t="inlineStr">
         <is>
-          <t>love, romance, devotion, affection</t>
+          <t>romance, devotion, divine love, affection, longing</t>
         </is>
       </c>
       <c r="D109" s="2" t="inlineStr"/>
@@ -2687,7 +2679,7 @@
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>reason, passions, judgment, hatred, emotions, feelings, mind, anger</t>
+          <t>passions, reason, judgment, anger, feelings, hatred</t>
         </is>
       </c>
       <c r="D110" s="2" t="inlineStr"/>
@@ -2705,7 +2697,7 @@
       </c>
       <c r="C111" s="2" t="inlineStr">
         <is>
-          <t>nature, universe, cosmos, the natural world</t>
+          <t>cosmos, the natural world, atoms, Tao, seasons</t>
         </is>
       </c>
       <c r="D111" s="2" t="inlineStr"/>
@@ -2723,7 +2715,7 @@
       </c>
       <c r="C112" s="2" t="inlineStr">
         <is>
-          <t>purpose, meaning, calling, meaning of life</t>
+          <t>meaning of life, calling, vocation, why live, nihilism</t>
         </is>
       </c>
       <c r="D112" s="2" t="inlineStr"/>
@@ -2741,7 +2733,7 @@
       </c>
       <c r="C113" s="2" t="inlineStr">
         <is>
-          <t>self-knowledge, know thyself, introspection, self-examination</t>
+          <t>know thyself, introspection, self-examination, the unexamined life, masks</t>
         </is>
       </c>
       <c r="D113" s="2" t="inlineStr"/>
@@ -2759,7 +2751,7 @@
       </c>
       <c r="C114" s="2" t="inlineStr">
         <is>
-          <t>solitude, stillness, silence, being alone</t>
+          <t>silence, being alone, retreat, quiet, hermit</t>
         </is>
       </c>
       <c r="D114" s="2" t="inlineStr"/>
@@ -2777,7 +2769,7 @@
       </c>
       <c r="C115" s="2" t="inlineStr">
         <is>
-          <t>suffering, resilience, pain, adversity, hardship</t>
+          <t>pain, adversity, hardship, consolation, grief</t>
         </is>
       </c>
       <c r="D115" s="2" t="inlineStr"/>
@@ -2793,11 +2785,7 @@
           <t>The self and the soul</t>
         </is>
       </c>
-      <c r="C116" s="2" t="inlineStr">
-        <is>
-          <t>the lower self</t>
-        </is>
-      </c>
+      <c r="C116" s="2" t="n"/>
       <c r="D116" s="2" t="inlineStr"/>
     </row>
     <row r="117">
@@ -2813,7 +2801,7 @@
       </c>
       <c r="C117" s="2" t="inlineStr">
         <is>
-          <t>time, the present moment, now, past and future</t>
+          <t>present moment, carpe diem, past and future, memory, the moment</t>
         </is>
       </c>
       <c r="D117" s="2" t="inlineStr"/>
@@ -2831,7 +2819,7 @@
       </c>
       <c r="C118" s="2" t="inlineStr">
         <is>
-          <t>prejudice, tolerance, intolerance, diversity, religious freedom</t>
+          <t>prejudice, intolerance, diversity, religious freedom, toleration</t>
         </is>
       </c>
       <c r="D118" s="2" t="inlineStr"/>
@@ -2849,7 +2837,7 @@
       </c>
       <c r="C119" s="2" t="inlineStr">
         <is>
-          <t>war, peace, violence, conflict</t>
+          <t>violence, conflict, nonviolence, revenge</t>
         </is>
       </c>
       <c r="D119" s="2" t="inlineStr"/>
@@ -2867,7 +2855,7 @@
       </c>
       <c r="C120" s="2" t="inlineStr">
         <is>
-          <t>work, action, effort, doing</t>
+          <t>effort, doing, karma yoga, wu wei, labour</t>
         </is>
       </c>
       <c r="D120" s="2" t="inlineStr"/>
@@ -2885,7 +2873,7 @@
       </c>
       <c r="C121" s="2" t="inlineStr">
         <is>
-          <t>wealth, money, poverty, riches, work</t>
+          <t>money, poverty, riches, labour, possessions</t>
         </is>
       </c>
       <c r="D121" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
The Library: thinkers, texts, paths, eras, and themes (120 pages, all Ready) with search, a weekly highlight, maps and timelines (Asia map, Rome's own dot, the thinkers through time), and ways in from cards, Past thoughts, and monthly questions; built and checked by tools/build_pages.py; new bottom bar (About moves to the Library and Settings); tour: "Where it comes from" card and a sentence on monthly questions; source links fixed (Seneca, Zhuangzi, Bhagavad Gita); Königsberg and Danzig with today's names
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/page-tags.xlsx
+++ b/content/page-tags.xlsx
@@ -1685,12 +1685,12 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>thinker-kakuzo-okakura</t>
+          <t>thinker-okakura-kakuzo</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>Kakuzo Okakura</t>
+          <t>Okakura Kakuzō</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
@@ -1700,7 +1700,7 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>Okakura Kakuzō, Okakura Tenshin, Okakura</t>
+          <t>Kakuzo Okakura, Okakura Tenshin, Okakura</t>
         </is>
       </c>
     </row>

</xml_diff>